<commit_message>
Fix cart paths, auth API proxy, and secure contact form
</commit_message>
<xml_diff>
--- a/products/Price List.xlsx
+++ b/products/Price List.xlsx
@@ -798,19 +798,19 @@
       </c>
     </row>
     <row r="20" ht="14.25">
-      <c r="A20" s="4" t="s">
+      <c r="A20" s="2" t="s">
         <v>15</v>
       </c>
       <c r="B20" s="2">
-        <v>1.8899999999999999</v>
+        <v>2.8900000000000001</v>
       </c>
     </row>
     <row r="21" ht="14.25">
-      <c r="A21" s="4" t="s">
+      <c r="A21" s="2" t="s">
         <v>16</v>
       </c>
       <c r="B21" s="2">
-        <v>3.3500000000000001</v>
+        <v>3.79</v>
       </c>
     </row>
     <row r="22" ht="14.25">
@@ -826,27 +826,27 @@
       </c>
     </row>
     <row r="24" ht="14.25">
-      <c r="A24" s="4" t="s">
+      <c r="A24" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B24" s="2">
-        <v>6.4900000000000002</v>
+      <c r="B24">
+        <v>10.18</v>
       </c>
     </row>
     <row r="25" ht="14.25">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B25" s="2">
-        <v>6.4900000000000002</v>
+        <v>8.1199999999999992</v>
       </c>
     </row>
     <row r="26" ht="14.25">
       <c r="A26" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B26" s="2">
-        <v>6.4900000000000002</v>
+      <c r="B26" s="4">
+        <v>10.18</v>
       </c>
     </row>
     <row r="27" ht="14.25"/>
@@ -859,15 +859,15 @@
       </c>
     </row>
     <row r="29" ht="14.25">
-      <c r="A29" s="4" t="s">
+      <c r="A29" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="B29" s="2">
+      <c r="B29">
         <v>27.539999999999999</v>
       </c>
     </row>
     <row r="30" ht="14.25">
-      <c r="A30" s="4" t="s">
+      <c r="A30" s="2" t="s">
         <v>23</v>
       </c>
       <c r="B30" s="2">

</xml_diff>